<commit_message>
modified the inpu template
</commit_message>
<xml_diff>
--- a/artifacts/input_template.xlsx
+++ b/artifacts/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\z0050s8t\Documents\rental-automation\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8EFFA7-A3FD-4E1B-981E-FA4DF09D8AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8417BC5-4EEB-4F57-9AA5-29A900EC862D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
   <si>
     <t>Field Name</t>
   </si>
@@ -95,22 +95,13 @@
     <t>Rent Per Sqft</t>
   </si>
   <si>
-    <t>Starting Monthly Rent</t>
-  </si>
-  <si>
     <t>Escalation %</t>
   </si>
   <si>
     <t>Escalation Frequency Months</t>
   </si>
   <si>
-    <t>Quoted CAM</t>
-  </si>
-  <si>
     <t>CAM Escalation %</t>
-  </si>
-  <si>
-    <t>CAM Escalation Frequency Months</t>
   </si>
   <si>
     <t>Billing Frequency</t>
@@ -125,25 +116,10 @@
     <t>Security Deposit Amount</t>
   </si>
   <si>
-    <t>Refundable Deposit</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Fitout Cost</t>
   </si>
   <si>
     <t>Useful Life Years</t>
-  </si>
-  <si>
-    <t>Residual Value</t>
-  </si>
-  <si>
-    <t>Discount Rate</t>
-  </si>
-  <si>
-    <t>Incremental Borrowing Rate</t>
   </si>
   <si>
     <t>Cost of Capital</t>
@@ -156,9 +132,6 @@
   </si>
   <si>
     <t>Imputed Interest Rate</t>
-  </si>
-  <si>
-    <t>Ready Reckoner Rate</t>
   </si>
   <si>
     <t>No. of 4 wheelers</t>
@@ -226,12 +199,21 @@
   <si>
     <t>Parking Escalation Frequency Months</t>
   </si>
+  <si>
+    <t>CAM per Sq ft</t>
+  </si>
+  <si>
+    <t>LEASE-001</t>
+  </si>
+  <si>
+    <t>Office</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -276,6 +258,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.9"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -330,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -350,6 +338,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -703,7 +694,9 @@
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
@@ -715,7 +708,9 @@
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
@@ -764,14 +759,16 @@
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="3"/>
+      <c r="B11" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="4">
-        <v>46113</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -779,7 +776,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="4">
-        <v>47938</v>
+        <v>48071</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -787,14 +784,17 @@
         <v>16</v>
       </c>
       <c r="B14" s="4">
-        <v>46113</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="3"/>
+      <c r="B15" s="3">
+        <f>(B13-B12)/365*12</f>
+        <v>60</v>
+      </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
@@ -812,148 +812,143 @@
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="3"/>
+      <c r="B18" s="5"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="5"/>
+      <c r="B19" s="6"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
-      <c r="B20" s="6"/>
+      <c r="B20" s="3" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
-        <v>23</v>
+      <c r="A21" s="2" t="s">
+        <v>25</v>
       </c>
-      <c r="B21">
-        <v>15.48</v>
+      <c r="B21" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
-        <v>24</v>
+      <c r="A22" s="2" t="s">
+        <v>26</v>
       </c>
-      <c r="B22">
-        <v>0.05</v>
-      </c>
+      <c r="B22" s="7"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
-        <v>25</v>
+      <c r="A23" s="2" t="s">
+        <v>27</v>
       </c>
-      <c r="B23">
-        <v>12</v>
-      </c>
+      <c r="B23" s="3"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>27</v>
+      <c r="B24" s="3">
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
-      <c r="B25" s="3">
-        <v>6</v>
+      <c r="B25" s="16">
+        <v>0.05</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
-      <c r="B26" s="7">
-        <v>11418000</v>
+      <c r="B26" s="3">
+        <v>12</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>31</v>
+      <c r="B27" s="3">
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
-        <v>32</v>
+      <c r="A28" s="8" t="s">
+        <v>29</v>
       </c>
-      <c r="B28" s="3"/>
+      <c r="B28" s="9">
+        <v>0.105</v>
+      </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B29" s="3">
-        <v>5</v>
+      <c r="A29" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="12"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="9">
+        <v>7.1099999999999997E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
+      <c r="A33" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B31" s="5"/>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" s="5"/>
-    </row>
-    <row r="33" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A33" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="9"/>
     </row>
     <row r="34" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A35" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35" s="12">
-        <v>500000</v>
+      <c r="A35" s="10" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="36" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A36" s="14" t="s">
-        <v>40</v>
+      <c r="A36" s="10" t="s">
+        <v>53</v>
       </c>
-      <c r="B36" s="9">
-        <v>7.1099999999999997E-2</v>
+      <c r="B36" s="17">
+        <v>0.15</v>
       </c>
     </row>
     <row r="37" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A37" s="14" t="s">
-        <v>41</v>
+      <c r="A37" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="B37">
-        <v>15000</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A38" s="10" t="s">
-        <v>42</v>
+      <c r="A38" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>110.5</v>
       </c>
       <c r="C38" s="10"/>
       <c r="E38" s="10"/>
@@ -9148,8 +9143,8 @@
       <c r="XFC38" s="10"/>
     </row>
     <row r="39" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
-        <v>43</v>
+      <c r="A39" s="15" t="s">
+        <v>38</v>
       </c>
       <c r="C39" s="10"/>
       <c r="E39" s="10"/>
@@ -17344,8 +17339,8 @@
       <c r="XFC39" s="10"/>
     </row>
     <row r="40" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A40" s="10" t="s">
-        <v>44</v>
+      <c r="A40" s="15" t="s">
+        <v>39</v>
       </c>
       <c r="C40" s="10"/>
       <c r="E40" s="10"/>
@@ -25540,8 +25535,8 @@
       <c r="XFC40" s="10"/>
     </row>
     <row r="41" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A41" s="10" t="s">
-        <v>45</v>
+      <c r="A41" s="15" t="s">
+        <v>40</v>
       </c>
       <c r="C41" s="10"/>
       <c r="E41" s="10"/>
@@ -33736,8 +33731,8 @@
       <c r="XFC41" s="10"/>
     </row>
     <row r="42" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A42" s="10" t="s">
-        <v>62</v>
+      <c r="A42" s="15" t="s">
+        <v>41</v>
       </c>
       <c r="C42" s="10"/>
       <c r="E42" s="10"/>
@@ -41932,8 +41927,8 @@
       <c r="XFC42" s="10"/>
     </row>
     <row r="43" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A43" s="10" t="s">
-        <v>63</v>
+      <c r="A43" s="15" t="s">
+        <v>42</v>
       </c>
       <c r="C43" s="10"/>
       <c r="E43" s="10"/>
@@ -50128,91 +50123,76 @@
       <c r="XFC43" s="10"/>
     </row>
     <row r="44" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A44" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B44">
-        <v>110.5</v>
+      <c r="A44" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A45" s="14" t="s">
+      <c r="A45" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
+      <c r="A46" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
+      <c r="A47" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
+      <c r="A48" s="15" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A46" s="14" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="15" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="47" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A47" s="14" t="s">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" s="15" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:1023 1025:2047 2049:3071 3073:4095 4097:5119 5121:6143 6145:7167 7169:8191 8193:9215 9217:10239 10241:11263 11265:12287 12289:13311 13313:14335 14337:15359 15361:16383" x14ac:dyDescent="0.35">
-      <c r="A48" s="14" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" s="15" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" s="14" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" s="15" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" s="14" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" s="15" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A51" s="14" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A52" s="14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A53" s="14" t="s">
-        <v>55</v>
-      </c>
-    </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A54" s="14" t="s">
-        <v>56</v>
-      </c>
+      <c r="A54" s="14"/>
       <c r="B54" s="13"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A55" s="14" t="s">
-        <v>57</v>
-      </c>
+      <c r="A55" s="14"/>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A56" s="14" t="s">
-        <v>58</v>
-      </c>
+      <c r="A56" s="14"/>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A57" s="14" t="s">
-        <v>59</v>
-      </c>
+      <c r="A57" s="14"/>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A58" s="14" t="s">
-        <v>60</v>
-      </c>
+      <c r="A58" s="14"/>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A59" s="14" t="s">
-        <v>61</v>
-      </c>
+      <c r="A59" s="14"/>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="B20" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>

</xml_diff>